<commit_message>
Added some sprite descriptions
</commit_message>
<xml_diff>
--- a/Notes/Items Brainstorming 2.xlsx
+++ b/Notes/Items Brainstorming 2.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Byron\Documents\GitHub\i_love_vampires\Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EBF0767-9351-467C-BDE1-2AC1C0B30C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6725274-BB7C-4302-9F38-501E252E3458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7560" yWindow="0" windowWidth="14196" windowHeight="12240" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="15" r:id="rId1"/>
     <sheet name="Template" sheetId="14" r:id="rId2"/>
     <sheet name="Notes" sheetId="10" r:id="rId3"/>
-    <sheet name="Light" sheetId="13" r:id="rId4"/>
-    <sheet name="Electricity" sheetId="11" r:id="rId5"/>
-    <sheet name="Ice" sheetId="8" r:id="rId6"/>
-    <sheet name="Fire" sheetId="1" r:id="rId7"/>
-    <sheet name="Boom" sheetId="3" r:id="rId8"/>
-    <sheet name="Military" sheetId="4" r:id="rId9"/>
-    <sheet name="Blood" sheetId="6" r:id="rId10"/>
+    <sheet name="Electricity" sheetId="11" r:id="rId4"/>
+    <sheet name="Ice" sheetId="8" r:id="rId5"/>
+    <sheet name="Fire" sheetId="1" r:id="rId6"/>
+    <sheet name="Boom" sheetId="3" r:id="rId7"/>
+    <sheet name="Military" sheetId="4" r:id="rId8"/>
+    <sheet name="Blood" sheetId="6" r:id="rId9"/>
+    <sheet name="Light" sheetId="13" r:id="rId10"/>
     <sheet name="Dark" sheetId="7" r:id="rId11"/>
     <sheet name="Poison" sheetId="5" r:id="rId12"/>
   </sheets>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="256">
   <si>
     <t>Set</t>
   </si>
@@ -837,6 +837,30 @@
   </si>
   <si>
     <t>FOX COMPANION</t>
+  </si>
+  <si>
+    <t>Death</t>
+  </si>
+  <si>
+    <t>Reckoning</t>
+  </si>
+  <si>
+    <t>Ultimate passive</t>
+  </si>
+  <si>
+    <t>ALL combatants are executed at 20% HP</t>
+  </si>
+  <si>
+    <t>Mortality</t>
+  </si>
+  <si>
+    <t>Aging</t>
+  </si>
+  <si>
+    <t>Passive</t>
+  </si>
+  <si>
+    <t>Enemies take more damage the longer they've been alive</t>
   </si>
 </sst>
 </file>
@@ -1206,440 +1230,353 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ECD360A-5E57-4978-B1EE-38123FDEACD9}">
-  <dimension ref="A1:S14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9ABB95F-2061-47FF-A70C-6E6F19379B05}">
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" customWidth="1"/>
+    <col min="6" max="6" width="37.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F1" t="s">
+        <v>217</v>
+      </c>
+      <c r="I1" t="s">
+        <v>224</v>
+      </c>
+      <c r="L1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" t="s">
+        <v>225</v>
+      </c>
+      <c r="L3" t="s">
+        <v>42</v>
+      </c>
+      <c r="M3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>214</v>
+      </c>
+      <c r="F8" t="s">
+        <v>220</v>
+      </c>
+      <c r="I8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" t="s">
+        <v>215</v>
+      </c>
+      <c r="F9" t="s">
+        <v>146</v>
+      </c>
+      <c r="I9" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>216</v>
+      </c>
+      <c r="F10" t="s">
+        <v>219</v>
+      </c>
+      <c r="I10" t="s">
+        <v>227</v>
+      </c>
+      <c r="L10" t="s">
+        <v>233</v>
+      </c>
+      <c r="M10" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="F11" t="s">
+        <v>221</v>
+      </c>
+      <c r="I11" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="F12" t="s">
+        <v>222</v>
+      </c>
+      <c r="I12" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="F13" t="s">
+        <v>223</v>
+      </c>
+      <c r="I13" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I14" t="s">
+        <v>231</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6027AA-2CD4-4903-A89B-F906149A51A3}">
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.6640625" customWidth="1"/>
     <col min="6" max="6" width="37.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>112</v>
-      </c>
-      <c r="C1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D1" t="s">
-        <v>112</v>
-      </c>
-      <c r="G1" t="s">
-        <v>112</v>
-      </c>
-      <c r="J1" t="s">
-        <v>112</v>
-      </c>
-      <c r="M1" t="s">
-        <v>112</v>
-      </c>
-      <c r="N1" t="s">
         <v>141</v>
       </c>
-      <c r="P1" t="s">
-        <v>112</v>
-      </c>
-      <c r="S1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="E1" t="s">
+        <v>141</v>
+      </c>
+      <c r="H1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C2" t="s">
-        <v>116</v>
-      </c>
-      <c r="D2" t="s">
-        <v>121</v>
-      </c>
-      <c r="G2" t="s">
-        <v>128</v>
+        <v>142</v>
+      </c>
+      <c r="E2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H2" t="s">
+        <v>147</v>
+      </c>
+      <c r="I2" t="s">
+        <v>248</v>
       </c>
       <c r="J2" t="s">
-        <v>135</v>
-      </c>
-      <c r="M2" t="s">
-        <v>149</v>
-      </c>
-      <c r="N2" t="s">
-        <v>142</v>
-      </c>
-      <c r="P2" t="s">
-        <v>181</v>
-      </c>
-      <c r="S2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C3" t="s">
-        <v>234</v>
+        <v>143</v>
+      </c>
+      <c r="I3" t="s">
+        <v>249</v>
       </c>
       <c r="J3" t="s">
-        <v>136</v>
-      </c>
-      <c r="M3" t="s">
-        <v>150</v>
-      </c>
-      <c r="N3" t="s">
-        <v>143</v>
-      </c>
-      <c r="S3" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>20</v>
       </c>
       <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
         <v>42</v>
       </c>
-      <c r="C4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>12</v>
+      <c r="I4" t="s">
+        <v>250</v>
       </c>
       <c r="J4" t="s">
-        <v>12</v>
-      </c>
-      <c r="M4" t="s">
-        <v>42</v>
-      </c>
-      <c r="N4" t="s">
-        <v>12</v>
-      </c>
-      <c r="P4" t="s">
-        <v>12</v>
-      </c>
-      <c r="S4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="D5" t="s">
-        <v>62</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="J5" t="s">
-        <v>14</v>
-      </c>
-      <c r="N5" t="s">
-        <v>14</v>
-      </c>
-      <c r="P5" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="E5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G6" t="s">
-        <v>62</v>
-      </c>
-      <c r="J6" t="s">
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
         <v>28</v>
       </c>
-      <c r="N6" t="s">
-        <v>27</v>
-      </c>
-      <c r="P6" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2</v>
       </c>
-      <c r="D7" t="s">
-        <v>122</v>
-      </c>
-      <c r="G7" t="s">
-        <v>129</v>
-      </c>
-      <c r="J7" t="s">
-        <v>137</v>
-      </c>
-      <c r="N7" t="s">
+      <c r="B7" t="s">
         <v>99</v>
       </c>
-      <c r="P7" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="G8" t="s">
-        <v>132</v>
-      </c>
-      <c r="J8" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
-      <c r="D9" t="s">
-        <v>123</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="B9" t="s">
         <v>101</v>
       </c>
-      <c r="N9" t="s">
-        <v>101</v>
-      </c>
-      <c r="P9" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>5</v>
       </c>
-      <c r="D10" t="s">
-        <v>124</v>
-      </c>
-      <c r="G10" t="s">
-        <v>130</v>
-      </c>
-      <c r="N10" t="s">
+      <c r="B10" t="s">
         <v>144</v>
       </c>
-      <c r="P10" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>115</v>
-      </c>
-      <c r="C11" t="s">
-        <v>117</v>
-      </c>
-      <c r="D11" t="s">
-        <v>125</v>
-      </c>
-      <c r="G11" t="s">
-        <v>131</v>
-      </c>
-      <c r="J11" t="s">
-        <v>139</v>
-      </c>
-      <c r="M11" t="s">
-        <v>151</v>
-      </c>
-      <c r="N11" t="s">
-        <v>134</v>
-      </c>
-      <c r="P11" t="s">
-        <v>187</v>
-      </c>
-      <c r="S11" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="C12" t="s">
-        <v>118</v>
-      </c>
-      <c r="D12" t="s">
-        <v>126</v>
-      </c>
-      <c r="G12" t="s">
-        <v>133</v>
-      </c>
-      <c r="J12" t="s">
-        <v>140</v>
-      </c>
-      <c r="S12" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="C13" t="s">
-        <v>119</v>
-      </c>
-      <c r="D13" t="s">
-        <v>127</v>
-      </c>
-      <c r="G13" t="s">
-        <v>134</v>
-      </c>
-      <c r="S13" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="C14" t="s">
-        <v>120</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6027AA-2CD4-4903-A89B-F906149A51A3}">
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1"/>
-    <col min="6" max="6" width="37.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E1" t="s">
-        <v>141</v>
-      </c>
-      <c r="H1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>142</v>
-      </c>
-      <c r="E2" t="s">
-        <v>145</v>
-      </c>
-      <c r="H2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s">
-        <v>99</v>
-      </c>
-      <c r="E7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
-        <v>101</v>
-      </c>
-      <c r="E9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" t="s">
-        <v>144</v>
-      </c>
-      <c r="E10" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" t="s">
         <v>134</v>
       </c>
       <c r="H11" t="s">
         <v>148</v>
+      </c>
+      <c r="I11" t="s">
+        <v>251</v>
+      </c>
+      <c r="J11" t="s">
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -1942,202 +1879,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9ABB95F-2061-47FF-A70C-6E6F19379B05}">
-  <dimension ref="A1:M14"/>
-  <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" customWidth="1"/>
-    <col min="6" max="6" width="37.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B1" t="s">
-        <v>209</v>
-      </c>
-      <c r="C1" t="s">
-        <v>212</v>
-      </c>
-      <c r="F1" t="s">
-        <v>217</v>
-      </c>
-      <c r="I1" t="s">
-        <v>224</v>
-      </c>
-      <c r="L1" t="s">
-        <v>232</v>
-      </c>
-      <c r="M1" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" t="s">
-        <v>225</v>
-      </c>
-      <c r="L3" t="s">
-        <v>42</v>
-      </c>
-      <c r="M3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F5" t="s">
-        <v>28</v>
-      </c>
-      <c r="I5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F7" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" t="s">
-        <v>214</v>
-      </c>
-      <c r="F8" t="s">
-        <v>220</v>
-      </c>
-      <c r="I8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" t="s">
-        <v>215</v>
-      </c>
-      <c r="F9" t="s">
-        <v>146</v>
-      </c>
-      <c r="I9" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" t="s">
-        <v>216</v>
-      </c>
-      <c r="F10" t="s">
-        <v>219</v>
-      </c>
-      <c r="I10" t="s">
-        <v>227</v>
-      </c>
-      <c r="L10" t="s">
-        <v>233</v>
-      </c>
-      <c r="M10" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="F11" t="s">
-        <v>221</v>
-      </c>
-      <c r="I11" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="F12" t="s">
-        <v>222</v>
-      </c>
-      <c r="I12" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="F13" t="s">
-        <v>223</v>
-      </c>
-      <c r="I13" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="I14" t="s">
-        <v>231</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CFCAA3D-8D96-40E1-8342-364E837A0F99}">
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2295,7 +2036,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3B61813-491F-482D-93BB-6CA7EB9EEB8B}">
   <dimension ref="A1:AW13"/>
   <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2489,7 +2230,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I13"/>
   <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2725,7 +2466,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECB25C07-9702-471D-A29D-72F8ADD9DDB6}">
   <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3012,7 +2753,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5E0E86E-176F-4A40-ADA4-26CB81CDF251}">
   <dimension ref="A1:BO15"/>
   <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3442,4 +3183,311 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ECD360A-5E57-4978-B1EE-38123FDEACD9}">
+  <dimension ref="A1:S14"/>
+  <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="6" max="6" width="37.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J1" t="s">
+        <v>112</v>
+      </c>
+      <c r="M1" t="s">
+        <v>112</v>
+      </c>
+      <c r="N1" t="s">
+        <v>141</v>
+      </c>
+      <c r="P1" t="s">
+        <v>112</v>
+      </c>
+      <c r="S1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G2" t="s">
+        <v>128</v>
+      </c>
+      <c r="J2" t="s">
+        <v>135</v>
+      </c>
+      <c r="M2" t="s">
+        <v>149</v>
+      </c>
+      <c r="N2" t="s">
+        <v>142</v>
+      </c>
+      <c r="P2" t="s">
+        <v>181</v>
+      </c>
+      <c r="S2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" t="s">
+        <v>234</v>
+      </c>
+      <c r="J3" t="s">
+        <v>136</v>
+      </c>
+      <c r="M3" t="s">
+        <v>150</v>
+      </c>
+      <c r="N3" t="s">
+        <v>143</v>
+      </c>
+      <c r="S3" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" t="s">
+        <v>12</v>
+      </c>
+      <c r="M4" t="s">
+        <v>42</v>
+      </c>
+      <c r="N4" t="s">
+        <v>12</v>
+      </c>
+      <c r="P4" t="s">
+        <v>12</v>
+      </c>
+      <c r="S4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N5" t="s">
+        <v>14</v>
+      </c>
+      <c r="P5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" t="s">
+        <v>62</v>
+      </c>
+      <c r="J6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P6" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>122</v>
+      </c>
+      <c r="G7" t="s">
+        <v>129</v>
+      </c>
+      <c r="J7" t="s">
+        <v>137</v>
+      </c>
+      <c r="N7" t="s">
+        <v>99</v>
+      </c>
+      <c r="P7" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" t="s">
+        <v>132</v>
+      </c>
+      <c r="J8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" t="s">
+        <v>123</v>
+      </c>
+      <c r="G9" t="s">
+        <v>101</v>
+      </c>
+      <c r="N9" t="s">
+        <v>101</v>
+      </c>
+      <c r="P9" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>124</v>
+      </c>
+      <c r="G10" t="s">
+        <v>130</v>
+      </c>
+      <c r="N10" t="s">
+        <v>144</v>
+      </c>
+      <c r="P10" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" t="s">
+        <v>125</v>
+      </c>
+      <c r="G11" t="s">
+        <v>131</v>
+      </c>
+      <c r="J11" t="s">
+        <v>139</v>
+      </c>
+      <c r="M11" t="s">
+        <v>151</v>
+      </c>
+      <c r="N11" t="s">
+        <v>134</v>
+      </c>
+      <c r="P11" t="s">
+        <v>187</v>
+      </c>
+      <c r="S11" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D12" t="s">
+        <v>126</v>
+      </c>
+      <c r="G12" t="s">
+        <v>133</v>
+      </c>
+      <c r="J12" t="s">
+        <v>140</v>
+      </c>
+      <c r="S12" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" t="s">
+        <v>127</v>
+      </c>
+      <c r="G13" t="s">
+        <v>134</v>
+      </c>
+      <c r="S13" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Compiler errors driving me crazy
Once you've fixed the problem remember to remove the extra constructors (including default constructors) if you don't need them
</commit_message>
<xml_diff>
--- a/Notes/Items Brainstorming 2.xlsx
+++ b/Notes/Items Brainstorming 2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Byron\Documents\GitHub\i_love_vampires\Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6725274-BB7C-4302-9F38-501E252E3458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D804A5-1664-4B58-B658-BD18AFE24952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7560" yWindow="0" windowWidth="14196" windowHeight="12240" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7560" yWindow="0" windowWidth="14196" windowHeight="12240" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="15" r:id="rId1"/>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="258">
   <si>
     <t>Set</t>
   </si>
@@ -861,6 +861,12 @@
   </si>
   <si>
     <t>Enemies take more damage the longer they've been alive</t>
+  </si>
+  <si>
+    <t>Divine Protection</t>
+  </si>
+  <si>
+    <t>When you dash into an attack effect, heal and destroy the effect. (parry)</t>
   </si>
 </sst>
 </file>
@@ -1231,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9ABB95F-2061-47FF-A70C-6E6F19379B05}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultColWidth="19.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.6640625" customWidth="1"/>
@@ -1239,7 +1245,7 @@
     <col min="6" max="6" width="37.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -1261,8 +1267,11 @@
       <c r="M1" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1271,7 +1280,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1291,7 +1300,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1305,7 +1314,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -1319,7 +1328,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1333,7 +1342,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1341,7 +1350,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1355,7 +1364,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1369,7 +1378,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -1388,8 +1397,11 @@
       <c r="M10" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N10" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
         <v>221</v>
       </c>
@@ -1397,7 +1409,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
         <v>222</v>
       </c>
@@ -1405,7 +1417,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
         <v>223</v>
       </c>
@@ -1413,7 +1425,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="I14" t="s">
         <v>231</v>
       </c>

</xml_diff>